<commit_message>
v10: slide-style Dashboard page and project start / end dates
- project_dashboard.aspx ("Dashboard" in every menu): five slides (Summary, Money,
  Effort / FTE, Value, project list) for a date range and / or a multi-select of
  projects; choice kept in the link and the browser; present full screen; print
  one slide per landscape page. Inline SVG charts, no new library.
- Register gains StartDate / EndDate (02 upgrade block, 08 backfill for the
  imported project list), captured on Registration Basics, the Excel template,
  the CSV import (now 34 columns) and shown in the report detail and CSV.
- API: projects&lite=1 returns the register without saved estimates.
- Docs: deployment order (run 02 or 08 before the new build), README, review.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bi8jGZngCKmVvuqhjQxHzc
</commit_message>
<xml_diff>
--- a/SW_CostModel/database/templates/projects-template.xlsx
+++ b/SW_CostModel/database/templates/projects-template.xlsx
@@ -150,6 +150,8 @@
     <col min="30" max="30" width="14" customWidth="1"/>
     <col min="31" max="31" width="14" customWidth="1"/>
     <col min="32" max="32" width="22" customWidth="1"/>
+    <col min="33" max="33" width="22" customWidth="1"/>
+    <col min="34" max="34" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -313,6 +315,16 @@
           <t xml:space="preserve">Note</t>
         </is>
       </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Start date</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">End date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -467,6 +479,16 @@
         </is>
       </c>
       <c r="AF2" s="4"/>
+      <c r="AG2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dd/mm/yyyy</t>
+        </is>
+      </c>
+      <c r="AH2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dd/mm/yyyy; empty = running</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2"/>
@@ -501,6 +523,8 @@
       <c r="AD3" s="7"/>
       <c r="AE3" s="7"/>
       <c r="AF3" s="2"/>
+      <c r="AG3" s="2"/>
+      <c r="AH3" s="2"/>
     </row>
     <row r="4">
       <c r="A4" s="2"/>
@@ -535,6 +559,8 @@
       <c r="AD4" s="7"/>
       <c r="AE4" s="7"/>
       <c r="AF4" s="2"/>
+      <c r="AG4" s="2"/>
+      <c r="AH4" s="2"/>
     </row>
     <row r="5">
       <c r="A5" s="2"/>
@@ -569,6 +595,8 @@
       <c r="AD5" s="7"/>
       <c r="AE5" s="7"/>
       <c r="AF5" s="2"/>
+      <c r="AG5" s="2"/>
+      <c r="AH5" s="2"/>
     </row>
     <row r="6">
       <c r="A6" s="2"/>
@@ -603,6 +631,8 @@
       <c r="AD6" s="7"/>
       <c r="AE6" s="7"/>
       <c r="AF6" s="2"/>
+      <c r="AG6" s="2"/>
+      <c r="AH6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" s="2"/>
@@ -637,6 +667,8 @@
       <c r="AD7" s="7"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="2"/>
+      <c r="AG7" s="2"/>
+      <c r="AH7" s="2"/>
     </row>
     <row r="8">
       <c r="A8" s="2"/>
@@ -671,6 +703,8 @@
       <c r="AD8" s="7"/>
       <c r="AE8" s="7"/>
       <c r="AF8" s="2"/>
+      <c r="AG8" s="2"/>
+      <c r="AH8" s="2"/>
     </row>
     <row r="9">
       <c r="A9" s="2"/>
@@ -705,6 +739,8 @@
       <c r="AD9" s="7"/>
       <c r="AE9" s="7"/>
       <c r="AF9" s="2"/>
+      <c r="AG9" s="2"/>
+      <c r="AH9" s="2"/>
     </row>
     <row r="10">
       <c r="A10" s="2"/>
@@ -739,6 +775,8 @@
       <c r="AD10" s="7"/>
       <c r="AE10" s="7"/>
       <c r="AF10" s="2"/>
+      <c r="AG10" s="2"/>
+      <c r="AH10" s="2"/>
     </row>
     <row r="11">
       <c r="A11" s="2"/>
@@ -773,6 +811,8 @@
       <c r="AD11" s="7"/>
       <c r="AE11" s="7"/>
       <c r="AF11" s="2"/>
+      <c r="AG11" s="2"/>
+      <c r="AH11" s="2"/>
     </row>
     <row r="12">
       <c r="A12" s="2"/>
@@ -807,6 +847,8 @@
       <c r="AD12" s="7"/>
       <c r="AE12" s="7"/>
       <c r="AF12" s="2"/>
+      <c r="AG12" s="2"/>
+      <c r="AH12" s="2"/>
     </row>
     <row r="13">
       <c r="A13" s="2"/>
@@ -841,6 +883,8 @@
       <c r="AD13" s="7"/>
       <c r="AE13" s="7"/>
       <c r="AF13" s="2"/>
+      <c r="AG13" s="2"/>
+      <c r="AH13" s="2"/>
     </row>
     <row r="14">
       <c r="A14" s="2"/>
@@ -875,6 +919,8 @@
       <c r="AD14" s="7"/>
       <c r="AE14" s="7"/>
       <c r="AF14" s="2"/>
+      <c r="AG14" s="2"/>
+      <c r="AH14" s="2"/>
     </row>
     <row r="15">
       <c r="A15" s="2"/>
@@ -909,6 +955,8 @@
       <c r="AD15" s="7"/>
       <c r="AE15" s="7"/>
       <c r="AF15" s="2"/>
+      <c r="AG15" s="2"/>
+      <c r="AH15" s="2"/>
     </row>
     <row r="16">
       <c r="A16" s="2"/>
@@ -943,6 +991,8 @@
       <c r="AD16" s="7"/>
       <c r="AE16" s="7"/>
       <c r="AF16" s="2"/>
+      <c r="AG16" s="2"/>
+      <c r="AH16" s="2"/>
     </row>
     <row r="17">
       <c r="A17" s="2"/>
@@ -977,6 +1027,8 @@
       <c r="AD17" s="7"/>
       <c r="AE17" s="7"/>
       <c r="AF17" s="2"/>
+      <c r="AG17" s="2"/>
+      <c r="AH17" s="2"/>
     </row>
     <row r="18">
       <c r="A18" s="2"/>
@@ -1011,6 +1063,8 @@
       <c r="AD18" s="7"/>
       <c r="AE18" s="7"/>
       <c r="AF18" s="2"/>
+      <c r="AG18" s="2"/>
+      <c r="AH18" s="2"/>
     </row>
     <row r="19">
       <c r="A19" s="2"/>
@@ -1045,6 +1099,8 @@
       <c r="AD19" s="7"/>
       <c r="AE19" s="7"/>
       <c r="AF19" s="2"/>
+      <c r="AG19" s="2"/>
+      <c r="AH19" s="2"/>
     </row>
     <row r="20">
       <c r="A20" s="2"/>
@@ -1079,6 +1135,8 @@
       <c r="AD20" s="7"/>
       <c r="AE20" s="7"/>
       <c r="AF20" s="2"/>
+      <c r="AG20" s="2"/>
+      <c r="AH20" s="2"/>
     </row>
     <row r="21">
       <c r="A21" s="2"/>
@@ -1113,6 +1171,8 @@
       <c r="AD21" s="7"/>
       <c r="AE21" s="7"/>
       <c r="AF21" s="2"/>
+      <c r="AG21" s="2"/>
+      <c r="AH21" s="2"/>
     </row>
     <row r="22">
       <c r="A22" s="2"/>
@@ -1147,6 +1207,8 @@
       <c r="AD22" s="7"/>
       <c r="AE22" s="7"/>
       <c r="AF22" s="2"/>
+      <c r="AG22" s="2"/>
+      <c r="AH22" s="2"/>
     </row>
     <row r="23">
       <c r="A23" s="2"/>
@@ -1181,6 +1243,8 @@
       <c r="AD23" s="7"/>
       <c r="AE23" s="7"/>
       <c r="AF23" s="2"/>
+      <c r="AG23" s="2"/>
+      <c r="AH23" s="2"/>
     </row>
     <row r="24">
       <c r="A24" s="2"/>
@@ -1215,6 +1279,8 @@
       <c r="AD24" s="7"/>
       <c r="AE24" s="7"/>
       <c r="AF24" s="2"/>
+      <c r="AG24" s="2"/>
+      <c r="AH24" s="2"/>
     </row>
     <row r="25">
       <c r="A25" s="2"/>
@@ -1249,6 +1315,8 @@
       <c r="AD25" s="7"/>
       <c r="AE25" s="7"/>
       <c r="AF25" s="2"/>
+      <c r="AG25" s="2"/>
+      <c r="AH25" s="2"/>
     </row>
     <row r="26">
       <c r="A26" s="2"/>
@@ -1283,6 +1351,8 @@
       <c r="AD26" s="7"/>
       <c r="AE26" s="7"/>
       <c r="AF26" s="2"/>
+      <c r="AG26" s="2"/>
+      <c r="AH26" s="2"/>
     </row>
     <row r="27">
       <c r="A27" s="2"/>
@@ -1317,6 +1387,8 @@
       <c r="AD27" s="7"/>
       <c r="AE27" s="7"/>
       <c r="AF27" s="2"/>
+      <c r="AG27" s="2"/>
+      <c r="AH27" s="2"/>
     </row>
     <row r="28">
       <c r="A28" s="2"/>
@@ -1351,6 +1423,8 @@
       <c r="AD28" s="7"/>
       <c r="AE28" s="7"/>
       <c r="AF28" s="2"/>
+      <c r="AG28" s="2"/>
+      <c r="AH28" s="2"/>
     </row>
     <row r="29">
       <c r="A29" s="2"/>
@@ -1385,6 +1459,8 @@
       <c r="AD29" s="7"/>
       <c r="AE29" s="7"/>
       <c r="AF29" s="2"/>
+      <c r="AG29" s="2"/>
+      <c r="AH29" s="2"/>
     </row>
     <row r="30">
       <c r="A30" s="2"/>
@@ -1419,6 +1495,8 @@
       <c r="AD30" s="7"/>
       <c r="AE30" s="7"/>
       <c r="AF30" s="2"/>
+      <c r="AG30" s="2"/>
+      <c r="AH30" s="2"/>
     </row>
     <row r="31">
       <c r="A31" s="2"/>
@@ -1453,6 +1531,8 @@
       <c r="AD31" s="7"/>
       <c r="AE31" s="7"/>
       <c r="AF31" s="2"/>
+      <c r="AG31" s="2"/>
+      <c r="AH31" s="2"/>
     </row>
     <row r="32">
       <c r="A32" s="2"/>
@@ -1487,6 +1567,8 @@
       <c r="AD32" s="7"/>
       <c r="AE32" s="7"/>
       <c r="AF32" s="2"/>
+      <c r="AG32" s="2"/>
+      <c r="AH32" s="2"/>
     </row>
     <row r="33">
       <c r="A33" s="2"/>
@@ -1521,6 +1603,8 @@
       <c r="AD33" s="7"/>
       <c r="AE33" s="7"/>
       <c r="AF33" s="2"/>
+      <c r="AG33" s="2"/>
+      <c r="AH33" s="2"/>
     </row>
     <row r="34">
       <c r="A34" s="2"/>
@@ -1555,6 +1639,8 @@
       <c r="AD34" s="7"/>
       <c r="AE34" s="7"/>
       <c r="AF34" s="2"/>
+      <c r="AG34" s="2"/>
+      <c r="AH34" s="2"/>
     </row>
     <row r="35">
       <c r="A35" s="2"/>
@@ -1589,6 +1675,8 @@
       <c r="AD35" s="7"/>
       <c r="AE35" s="7"/>
       <c r="AF35" s="2"/>
+      <c r="AG35" s="2"/>
+      <c r="AH35" s="2"/>
     </row>
     <row r="36">
       <c r="A36" s="2"/>
@@ -1623,6 +1711,8 @@
       <c r="AD36" s="7"/>
       <c r="AE36" s="7"/>
       <c r="AF36" s="2"/>
+      <c r="AG36" s="2"/>
+      <c r="AH36" s="2"/>
     </row>
     <row r="37">
       <c r="A37" s="2"/>
@@ -1657,6 +1747,8 @@
       <c r="AD37" s="7"/>
       <c r="AE37" s="7"/>
       <c r="AF37" s="2"/>
+      <c r="AG37" s="2"/>
+      <c r="AH37" s="2"/>
     </row>
     <row r="38">
       <c r="A38" s="2"/>
@@ -1691,6 +1783,8 @@
       <c r="AD38" s="7"/>
       <c r="AE38" s="7"/>
       <c r="AF38" s="2"/>
+      <c r="AG38" s="2"/>
+      <c r="AH38" s="2"/>
     </row>
     <row r="39">
       <c r="A39" s="2"/>
@@ -1725,6 +1819,8 @@
       <c r="AD39" s="7"/>
       <c r="AE39" s="7"/>
       <c r="AF39" s="2"/>
+      <c r="AG39" s="2"/>
+      <c r="AH39" s="2"/>
     </row>
     <row r="40">
       <c r="A40" s="2"/>
@@ -1759,6 +1855,8 @@
       <c r="AD40" s="7"/>
       <c r="AE40" s="7"/>
       <c r="AF40" s="2"/>
+      <c r="AG40" s="2"/>
+      <c r="AH40" s="2"/>
     </row>
     <row r="41">
       <c r="A41" s="2"/>
@@ -1793,6 +1891,8 @@
       <c r="AD41" s="7"/>
       <c r="AE41" s="7"/>
       <c r="AF41" s="2"/>
+      <c r="AG41" s="2"/>
+      <c r="AH41" s="2"/>
     </row>
     <row r="42">
       <c r="A42" s="2"/>
@@ -1827,6 +1927,8 @@
       <c r="AD42" s="7"/>
       <c r="AE42" s="7"/>
       <c r="AF42" s="2"/>
+      <c r="AG42" s="2"/>
+      <c r="AH42" s="2"/>
     </row>
     <row r="43">
       <c r="A43" s="2"/>
@@ -1861,6 +1963,8 @@
       <c r="AD43" s="7"/>
       <c r="AE43" s="7"/>
       <c r="AF43" s="2"/>
+      <c r="AG43" s="2"/>
+      <c r="AH43" s="2"/>
     </row>
     <row r="44">
       <c r="A44" s="2"/>
@@ -1895,6 +1999,8 @@
       <c r="AD44" s="7"/>
       <c r="AE44" s="7"/>
       <c r="AF44" s="2"/>
+      <c r="AG44" s="2"/>
+      <c r="AH44" s="2"/>
     </row>
     <row r="45">
       <c r="A45" s="2"/>
@@ -1929,6 +2035,8 @@
       <c r="AD45" s="7"/>
       <c r="AE45" s="7"/>
       <c r="AF45" s="2"/>
+      <c r="AG45" s="2"/>
+      <c r="AH45" s="2"/>
     </row>
     <row r="46">
       <c r="A46" s="2"/>
@@ -1963,6 +2071,8 @@
       <c r="AD46" s="7"/>
       <c r="AE46" s="7"/>
       <c r="AF46" s="2"/>
+      <c r="AG46" s="2"/>
+      <c r="AH46" s="2"/>
     </row>
     <row r="47">
       <c r="A47" s="2"/>
@@ -1997,6 +2107,8 @@
       <c r="AD47" s="7"/>
       <c r="AE47" s="7"/>
       <c r="AF47" s="2"/>
+      <c r="AG47" s="2"/>
+      <c r="AH47" s="2"/>
     </row>
     <row r="48">
       <c r="A48" s="2"/>
@@ -2031,6 +2143,8 @@
       <c r="AD48" s="7"/>
       <c r="AE48" s="7"/>
       <c r="AF48" s="2"/>
+      <c r="AG48" s="2"/>
+      <c r="AH48" s="2"/>
     </row>
     <row r="49">
       <c r="A49" s="2"/>
@@ -2065,6 +2179,8 @@
       <c r="AD49" s="7"/>
       <c r="AE49" s="7"/>
       <c r="AF49" s="2"/>
+      <c r="AG49" s="2"/>
+      <c r="AH49" s="2"/>
     </row>
     <row r="50">
       <c r="A50" s="2"/>
@@ -2099,6 +2215,8 @@
       <c r="AD50" s="7"/>
       <c r="AE50" s="7"/>
       <c r="AF50" s="2"/>
+      <c r="AG50" s="2"/>
+      <c r="AH50" s="2"/>
     </row>
     <row r="51">
       <c r="A51" s="2"/>
@@ -2133,6 +2251,8 @@
       <c r="AD51" s="7"/>
       <c r="AE51" s="7"/>
       <c r="AF51" s="2"/>
+      <c r="AG51" s="2"/>
+      <c r="AH51" s="2"/>
     </row>
     <row r="52">
       <c r="A52" s="2"/>
@@ -2167,6 +2287,8 @@
       <c r="AD52" s="7"/>
       <c r="AE52" s="7"/>
       <c r="AF52" s="2"/>
+      <c r="AG52" s="2"/>
+      <c r="AH52" s="2"/>
     </row>
     <row r="53">
       <c r="A53" s="2"/>
@@ -2201,6 +2323,8 @@
       <c r="AD53" s="7"/>
       <c r="AE53" s="7"/>
       <c r="AF53" s="2"/>
+      <c r="AG53" s="2"/>
+      <c r="AH53" s="2"/>
     </row>
     <row r="54">
       <c r="A54" s="2"/>
@@ -2235,6 +2359,8 @@
       <c r="AD54" s="7"/>
       <c r="AE54" s="7"/>
       <c r="AF54" s="2"/>
+      <c r="AG54" s="2"/>
+      <c r="AH54" s="2"/>
     </row>
     <row r="55">
       <c r="A55" s="2"/>
@@ -2269,6 +2395,8 @@
       <c r="AD55" s="7"/>
       <c r="AE55" s="7"/>
       <c r="AF55" s="2"/>
+      <c r="AG55" s="2"/>
+      <c r="AH55" s="2"/>
     </row>
     <row r="56">
       <c r="A56" s="2"/>
@@ -2303,6 +2431,8 @@
       <c r="AD56" s="7"/>
       <c r="AE56" s="7"/>
       <c r="AF56" s="2"/>
+      <c r="AG56" s="2"/>
+      <c r="AH56" s="2"/>
     </row>
     <row r="57">
       <c r="A57" s="2"/>
@@ -2337,6 +2467,8 @@
       <c r="AD57" s="7"/>
       <c r="AE57" s="7"/>
       <c r="AF57" s="2"/>
+      <c r="AG57" s="2"/>
+      <c r="AH57" s="2"/>
     </row>
     <row r="58">
       <c r="A58" s="2"/>
@@ -2371,6 +2503,8 @@
       <c r="AD58" s="7"/>
       <c r="AE58" s="7"/>
       <c r="AF58" s="2"/>
+      <c r="AG58" s="2"/>
+      <c r="AH58" s="2"/>
     </row>
     <row r="59">
       <c r="A59" s="2"/>
@@ -2405,6 +2539,8 @@
       <c r="AD59" s="7"/>
       <c r="AE59" s="7"/>
       <c r="AF59" s="2"/>
+      <c r="AG59" s="2"/>
+      <c r="AH59" s="2"/>
     </row>
     <row r="60">
       <c r="A60" s="2"/>
@@ -2439,6 +2575,8 @@
       <c r="AD60" s="7"/>
       <c r="AE60" s="7"/>
       <c r="AF60" s="2"/>
+      <c r="AG60" s="2"/>
+      <c r="AH60" s="2"/>
     </row>
     <row r="61">
       <c r="A61" s="2"/>
@@ -2473,6 +2611,8 @@
       <c r="AD61" s="7"/>
       <c r="AE61" s="7"/>
       <c r="AF61" s="2"/>
+      <c r="AG61" s="2"/>
+      <c r="AH61" s="2"/>
     </row>
     <row r="62">
       <c r="A62" s="2"/>
@@ -2507,6 +2647,8 @@
       <c r="AD62" s="7"/>
       <c r="AE62" s="7"/>
       <c r="AF62" s="2"/>
+      <c r="AG62" s="2"/>
+      <c r="AH62" s="2"/>
     </row>
     <row r="63">
       <c r="A63" s="2"/>
@@ -2541,6 +2683,8 @@
       <c r="AD63" s="7"/>
       <c r="AE63" s="7"/>
       <c r="AF63" s="2"/>
+      <c r="AG63" s="2"/>
+      <c r="AH63" s="2"/>
     </row>
     <row r="64">
       <c r="A64" s="2"/>
@@ -2575,6 +2719,8 @@
       <c r="AD64" s="7"/>
       <c r="AE64" s="7"/>
       <c r="AF64" s="2"/>
+      <c r="AG64" s="2"/>
+      <c r="AH64" s="2"/>
     </row>
     <row r="65">
       <c r="A65" s="2"/>
@@ -2609,6 +2755,8 @@
       <c r="AD65" s="7"/>
       <c r="AE65" s="7"/>
       <c r="AF65" s="2"/>
+      <c r="AG65" s="2"/>
+      <c r="AH65" s="2"/>
     </row>
     <row r="66">
       <c r="A66" s="2"/>
@@ -2643,6 +2791,8 @@
       <c r="AD66" s="7"/>
       <c r="AE66" s="7"/>
       <c r="AF66" s="2"/>
+      <c r="AG66" s="2"/>
+      <c r="AH66" s="2"/>
     </row>
     <row r="67">
       <c r="A67" s="2"/>
@@ -2677,6 +2827,8 @@
       <c r="AD67" s="7"/>
       <c r="AE67" s="7"/>
       <c r="AF67" s="2"/>
+      <c r="AG67" s="2"/>
+      <c r="AH67" s="2"/>
     </row>
     <row r="68">
       <c r="A68" s="2"/>
@@ -2711,6 +2863,8 @@
       <c r="AD68" s="7"/>
       <c r="AE68" s="7"/>
       <c r="AF68" s="2"/>
+      <c r="AG68" s="2"/>
+      <c r="AH68" s="2"/>
     </row>
     <row r="69">
       <c r="A69" s="2"/>
@@ -2745,6 +2899,8 @@
       <c r="AD69" s="7"/>
       <c r="AE69" s="7"/>
       <c r="AF69" s="2"/>
+      <c r="AG69" s="2"/>
+      <c r="AH69" s="2"/>
     </row>
     <row r="70">
       <c r="A70" s="2"/>
@@ -2779,6 +2935,8 @@
       <c r="AD70" s="7"/>
       <c r="AE70" s="7"/>
       <c r="AF70" s="2"/>
+      <c r="AG70" s="2"/>
+      <c r="AH70" s="2"/>
     </row>
     <row r="71">
       <c r="A71" s="2"/>
@@ -2813,6 +2971,8 @@
       <c r="AD71" s="7"/>
       <c r="AE71" s="7"/>
       <c r="AF71" s="2"/>
+      <c r="AG71" s="2"/>
+      <c r="AH71" s="2"/>
     </row>
     <row r="72">
       <c r="A72" s="2"/>
@@ -2847,6 +3007,8 @@
       <c r="AD72" s="7"/>
       <c r="AE72" s="7"/>
       <c r="AF72" s="2"/>
+      <c r="AG72" s="2"/>
+      <c r="AH72" s="2"/>
     </row>
     <row r="73">
       <c r="A73" s="2"/>
@@ -2881,6 +3043,8 @@
       <c r="AD73" s="7"/>
       <c r="AE73" s="7"/>
       <c r="AF73" s="2"/>
+      <c r="AG73" s="2"/>
+      <c r="AH73" s="2"/>
     </row>
     <row r="74">
       <c r="A74" s="2"/>
@@ -2915,6 +3079,8 @@
       <c r="AD74" s="7"/>
       <c r="AE74" s="7"/>
       <c r="AF74" s="2"/>
+      <c r="AG74" s="2"/>
+      <c r="AH74" s="2"/>
     </row>
     <row r="75">
       <c r="A75" s="2"/>
@@ -2949,6 +3115,8 @@
       <c r="AD75" s="7"/>
       <c r="AE75" s="7"/>
       <c r="AF75" s="2"/>
+      <c r="AG75" s="2"/>
+      <c r="AH75" s="2"/>
     </row>
     <row r="76">
       <c r="A76" s="2"/>
@@ -2983,6 +3151,8 @@
       <c r="AD76" s="7"/>
       <c r="AE76" s="7"/>
       <c r="AF76" s="2"/>
+      <c r="AG76" s="2"/>
+      <c r="AH76" s="2"/>
     </row>
     <row r="77">
       <c r="A77" s="2"/>
@@ -3017,6 +3187,8 @@
       <c r="AD77" s="7"/>
       <c r="AE77" s="7"/>
       <c r="AF77" s="2"/>
+      <c r="AG77" s="2"/>
+      <c r="AH77" s="2"/>
     </row>
     <row r="78">
       <c r="A78" s="2"/>
@@ -3051,6 +3223,8 @@
       <c r="AD78" s="7"/>
       <c r="AE78" s="7"/>
       <c r="AF78" s="2"/>
+      <c r="AG78" s="2"/>
+      <c r="AH78" s="2"/>
     </row>
     <row r="79">
       <c r="A79" s="2"/>
@@ -3085,6 +3259,8 @@
       <c r="AD79" s="7"/>
       <c r="AE79" s="7"/>
       <c r="AF79" s="2"/>
+      <c r="AG79" s="2"/>
+      <c r="AH79" s="2"/>
     </row>
     <row r="80">
       <c r="A80" s="2"/>
@@ -3119,6 +3295,8 @@
       <c r="AD80" s="7"/>
       <c r="AE80" s="7"/>
       <c r="AF80" s="2"/>
+      <c r="AG80" s="2"/>
+      <c r="AH80" s="2"/>
     </row>
     <row r="81">
       <c r="A81" s="2"/>
@@ -3153,6 +3331,8 @@
       <c r="AD81" s="7"/>
       <c r="AE81" s="7"/>
       <c r="AF81" s="2"/>
+      <c r="AG81" s="2"/>
+      <c r="AH81" s="2"/>
     </row>
     <row r="82">
       <c r="A82" s="2"/>
@@ -3187,6 +3367,8 @@
       <c r="AD82" s="7"/>
       <c r="AE82" s="7"/>
       <c r="AF82" s="2"/>
+      <c r="AG82" s="2"/>
+      <c r="AH82" s="2"/>
     </row>
     <row r="83">
       <c r="A83" s="2"/>
@@ -3221,6 +3403,8 @@
       <c r="AD83" s="7"/>
       <c r="AE83" s="7"/>
       <c r="AF83" s="2"/>
+      <c r="AG83" s="2"/>
+      <c r="AH83" s="2"/>
     </row>
     <row r="84">
       <c r="A84" s="2"/>
@@ -3255,6 +3439,8 @@
       <c r="AD84" s="7"/>
       <c r="AE84" s="7"/>
       <c r="AF84" s="2"/>
+      <c r="AG84" s="2"/>
+      <c r="AH84" s="2"/>
     </row>
     <row r="85">
       <c r="A85" s="2"/>
@@ -3289,6 +3475,8 @@
       <c r="AD85" s="7"/>
       <c r="AE85" s="7"/>
       <c r="AF85" s="2"/>
+      <c r="AG85" s="2"/>
+      <c r="AH85" s="2"/>
     </row>
     <row r="86">
       <c r="A86" s="2"/>
@@ -3323,6 +3511,8 @@
       <c r="AD86" s="7"/>
       <c r="AE86" s="7"/>
       <c r="AF86" s="2"/>
+      <c r="AG86" s="2"/>
+      <c r="AH86" s="2"/>
     </row>
     <row r="87">
       <c r="A87" s="2"/>
@@ -3357,6 +3547,8 @@
       <c r="AD87" s="7"/>
       <c r="AE87" s="7"/>
       <c r="AF87" s="2"/>
+      <c r="AG87" s="2"/>
+      <c r="AH87" s="2"/>
     </row>
     <row r="88">
       <c r="A88" s="2"/>
@@ -3391,6 +3583,8 @@
       <c r="AD88" s="7"/>
       <c r="AE88" s="7"/>
       <c r="AF88" s="2"/>
+      <c r="AG88" s="2"/>
+      <c r="AH88" s="2"/>
     </row>
     <row r="89">
       <c r="A89" s="2"/>
@@ -3425,6 +3619,8 @@
       <c r="AD89" s="7"/>
       <c r="AE89" s="7"/>
       <c r="AF89" s="2"/>
+      <c r="AG89" s="2"/>
+      <c r="AH89" s="2"/>
     </row>
     <row r="90">
       <c r="A90" s="2"/>
@@ -3459,6 +3655,8 @@
       <c r="AD90" s="7"/>
       <c r="AE90" s="7"/>
       <c r="AF90" s="2"/>
+      <c r="AG90" s="2"/>
+      <c r="AH90" s="2"/>
     </row>
     <row r="91">
       <c r="A91" s="2"/>
@@ -3493,6 +3691,8 @@
       <c r="AD91" s="7"/>
       <c r="AE91" s="7"/>
       <c r="AF91" s="2"/>
+      <c r="AG91" s="2"/>
+      <c r="AH91" s="2"/>
     </row>
     <row r="92">
       <c r="A92" s="2"/>
@@ -3527,6 +3727,8 @@
       <c r="AD92" s="7"/>
       <c r="AE92" s="7"/>
       <c r="AF92" s="2"/>
+      <c r="AG92" s="2"/>
+      <c r="AH92" s="2"/>
     </row>
     <row r="93">
       <c r="A93" s="2"/>
@@ -3561,6 +3763,8 @@
       <c r="AD93" s="7"/>
       <c r="AE93" s="7"/>
       <c r="AF93" s="2"/>
+      <c r="AG93" s="2"/>
+      <c r="AH93" s="2"/>
     </row>
     <row r="94">
       <c r="A94" s="2"/>
@@ -3595,6 +3799,8 @@
       <c r="AD94" s="7"/>
       <c r="AE94" s="7"/>
       <c r="AF94" s="2"/>
+      <c r="AG94" s="2"/>
+      <c r="AH94" s="2"/>
     </row>
     <row r="95">
       <c r="A95" s="2"/>
@@ -3629,6 +3835,8 @@
       <c r="AD95" s="7"/>
       <c r="AE95" s="7"/>
       <c r="AF95" s="2"/>
+      <c r="AG95" s="2"/>
+      <c r="AH95" s="2"/>
     </row>
     <row r="96">
       <c r="A96" s="2"/>
@@ -3663,6 +3871,8 @@
       <c r="AD96" s="7"/>
       <c r="AE96" s="7"/>
       <c r="AF96" s="2"/>
+      <c r="AG96" s="2"/>
+      <c r="AH96" s="2"/>
     </row>
     <row r="97">
       <c r="A97" s="2"/>
@@ -3697,6 +3907,8 @@
       <c r="AD97" s="7"/>
       <c r="AE97" s="7"/>
       <c r="AF97" s="2"/>
+      <c r="AG97" s="2"/>
+      <c r="AH97" s="2"/>
     </row>
     <row r="98">
       <c r="A98" s="2"/>
@@ -3731,6 +3943,8 @@
       <c r="AD98" s="7"/>
       <c r="AE98" s="7"/>
       <c r="AF98" s="2"/>
+      <c r="AG98" s="2"/>
+      <c r="AH98" s="2"/>
     </row>
     <row r="99">
       <c r="A99" s="2"/>
@@ -3765,6 +3979,8 @@
       <c r="AD99" s="7"/>
       <c r="AE99" s="7"/>
       <c r="AF99" s="2"/>
+      <c r="AG99" s="2"/>
+      <c r="AH99" s="2"/>
     </row>
     <row r="100">
       <c r="A100" s="2"/>
@@ -3799,6 +4015,8 @@
       <c r="AD100" s="7"/>
       <c r="AE100" s="7"/>
       <c r="AF100" s="2"/>
+      <c r="AG100" s="2"/>
+      <c r="AH100" s="2"/>
     </row>
     <row r="101">
       <c r="A101" s="2"/>
@@ -3833,6 +4051,8 @@
       <c r="AD101" s="7"/>
       <c r="AE101" s="7"/>
       <c r="AF101" s="2"/>
+      <c r="AG101" s="2"/>
+      <c r="AH101" s="2"/>
     </row>
     <row r="102">
       <c r="A102" s="2"/>
@@ -3867,6 +4087,8 @@
       <c r="AD102" s="7"/>
       <c r="AE102" s="7"/>
       <c r="AF102" s="2"/>
+      <c r="AG102" s="2"/>
+      <c r="AH102" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="16">
@@ -3910,13 +4132,13 @@
       <formula1>Lists!$M$2:$M$3</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Choose from the list" error="Pick a value from the drop-down list." sqref="Y3:Y102">
-      <formula1>Lists!$N$2:$N$10</formula1>
+      <formula1>Lists!$N$2:$N$9</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Choose from the list" error="Pick a value from the drop-down list." sqref="AA3:AA102">
-      <formula1>Lists!$N$2:$N$10</formula1>
+      <formula1>Lists!$N$2:$N$9</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Choose from the list" error="Pick a value from the drop-down list." sqref="AC3:AC102">
-      <formula1>Lists!$N$2:$N$10</formula1>
+      <formula1>Lists!$N$2:$N$9</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4310,13 +4532,6 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="N10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Inventory reduced (₹)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>